<commit_message>
adding terms to the list of terms and fixing SDC2 import links
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations/ClimOO Ontology vocabulary - List.xlsx
+++ b/ClimOO material/materials for implementations/ClimOO Ontology vocabulary - List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AF2C40-E981-1E46-84B7-CF0CE48B75F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715DBAB1-FB88-EC4D-B3CC-45B045DE9E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33000" yWindow="1540" windowWidth="27640" windowHeight="16440" xr2:uid="{871EAFEC-93A1-F947-B348-9B49072C2753}"/>
+    <workbookView xWindow="42460" yWindow="1780" windowWidth="27640" windowHeight="16440" xr2:uid="{871EAFEC-93A1-F947-B348-9B49072C2753}"/>
   </bookViews>
   <sheets>
     <sheet name="ClimOO Vocabulary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="832">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1664" uniqueCount="837">
   <si>
     <t>entity</t>
   </si>
@@ -2532,6 +2532,21 @@
   </si>
   <si>
     <t>Not yet</t>
+  </si>
+  <si>
+    <t>alteration process of temperature</t>
+  </si>
+  <si>
+    <t>process of increase in UV irradiation</t>
+  </si>
+  <si>
+    <t>UV irradiation process</t>
+  </si>
+  <si>
+    <t>process of alteration in species types</t>
+  </si>
+  <si>
+    <t>process of increase in atmospheric CO2 and CO2-equivalent concentration</t>
   </si>
 </sst>
 </file>
@@ -2612,26 +2627,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2961,7 +2967,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B6896C0-3354-CF47-84D5-E5D7BD388021}">
-  <dimension ref="A1:E828"/>
+  <dimension ref="A1:E833"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="75.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -6473,7 +6479,7 @@
     </row>
     <row r="390" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A390" s="1"/>
-      <c r="B390" s="5" t="s">
+      <c r="B390" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C390" s="3"/>
@@ -6482,7 +6488,7 @@
       <c r="A391" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="B391" s="5" t="s">
+      <c r="B391" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C391" s="3"/>
@@ -6491,7 +6497,7 @@
       <c r="A392" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B392" s="5" t="s">
+      <c r="B392" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C392" s="3"/>
@@ -6500,7 +6506,7 @@
       <c r="A393" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="B393" s="5" t="s">
+      <c r="B393" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C393" s="3"/>
@@ -6509,7 +6515,7 @@
       <c r="A394" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="B394" s="5" t="s">
+      <c r="B394" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C394" s="3"/>
@@ -6518,7 +6524,7 @@
       <c r="A395" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="B395" s="5" t="s">
+      <c r="B395" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C395" s="3"/>
@@ -6527,7 +6533,7 @@
       <c r="A396" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B396" s="5" t="s">
+      <c r="B396" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C396" s="3"/>
@@ -6536,7 +6542,7 @@
       <c r="A397" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B397" s="5" t="s">
+      <c r="B397" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C397" s="3"/>
@@ -6545,7 +6551,7 @@
       <c r="A398" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="B398" s="5" t="s">
+      <c r="B398" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C398" s="3"/>
@@ -6554,7 +6560,7 @@
       <c r="A399" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="B399" s="5" t="s">
+      <c r="B399" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C399" s="3"/>
@@ -6563,7 +6569,7 @@
       <c r="A400" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B400" s="5" t="s">
+      <c r="B400" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C400" s="3"/>
@@ -6572,7 +6578,7 @@
       <c r="A401" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="B401" s="5" t="s">
+      <c r="B401" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C401" s="3"/>
@@ -6581,7 +6587,7 @@
       <c r="A402" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B402" s="5" t="s">
+      <c r="B402" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C402" s="3"/>
@@ -6590,7 +6596,7 @@
       <c r="A403" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="B403" s="5" t="s">
+      <c r="B403" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C403" s="3"/>
@@ -6599,7 +6605,7 @@
       <c r="A404" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B404" s="5" t="s">
+      <c r="B404" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C404" s="3"/>
@@ -6608,7 +6614,7 @@
       <c r="A405" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="B405" s="5" t="s">
+      <c r="B405" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C405" s="3"/>
@@ -6617,7 +6623,7 @@
       <c r="A406" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B406" s="5" t="s">
+      <c r="B406" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C406" s="3"/>
@@ -6626,7 +6632,7 @@
       <c r="A407" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="B407" s="5" t="s">
+      <c r="B407" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C407" s="3"/>
@@ -6635,7 +6641,7 @@
       <c r="A408" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B408" s="5" t="s">
+      <c r="B408" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C408" s="3"/>
@@ -6644,7 +6650,7 @@
       <c r="A409" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="B409" s="5" t="s">
+      <c r="B409" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C409" s="3"/>
@@ -6653,7 +6659,7 @@
       <c r="A410" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B410" s="5" t="s">
+      <c r="B410" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C410" s="3"/>
@@ -6662,7 +6668,7 @@
       <c r="A411" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="B411" s="5" t="s">
+      <c r="B411" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C411" s="3"/>
@@ -6671,7 +6677,7 @@
       <c r="A412" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B412" s="5" t="s">
+      <c r="B412" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C412" s="3"/>
@@ -6680,7 +6686,7 @@
       <c r="A413" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="B413" s="5" t="s">
+      <c r="B413" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C413" s="3"/>
@@ -6689,7 +6695,7 @@
       <c r="A414" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B414" s="5" t="s">
+      <c r="B414" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C414" s="3"/>
@@ -6698,7 +6704,7 @@
       <c r="A415" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="B415" s="5" t="s">
+      <c r="B415" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C415" s="3"/>
@@ -6707,7 +6713,7 @@
       <c r="A416" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B416" s="5" t="s">
+      <c r="B416" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C416" s="3"/>
@@ -6716,7 +6722,7 @@
       <c r="A417" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="B417" s="5" t="s">
+      <c r="B417" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C417" s="3"/>
@@ -6725,7 +6731,7 @@
       <c r="A418" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B418" s="5" t="s">
+      <c r="B418" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C418" s="3"/>
@@ -6734,7 +6740,7 @@
       <c r="A419" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="B419" s="5" t="s">
+      <c r="B419" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C419" s="3"/>
@@ -6743,7 +6749,7 @@
       <c r="A420" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="B420" s="5" t="s">
+      <c r="B420" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C420" s="3"/>
@@ -6752,7 +6758,7 @@
       <c r="A421" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="B421" s="5" t="s">
+      <c r="B421" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C421" s="3"/>
@@ -6761,7 +6767,7 @@
       <c r="A422" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B422" s="5" t="s">
+      <c r="B422" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C422" s="3"/>
@@ -6770,7 +6776,7 @@
       <c r="A423" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="B423" s="5" t="s">
+      <c r="B423" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C423" s="3"/>
@@ -6779,7 +6785,7 @@
       <c r="A424" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="B424" s="5" t="s">
+      <c r="B424" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C424" s="3"/>
@@ -6788,7 +6794,7 @@
       <c r="A425" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="B425" s="5" t="s">
+      <c r="B425" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C425" s="3"/>
@@ -6797,7 +6803,7 @@
       <c r="A426" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B426" s="5" t="s">
+      <c r="B426" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C426" s="3"/>
@@ -6806,7 +6812,7 @@
       <c r="A427" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="B427" s="5" t="s">
+      <c r="B427" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C427" s="3"/>
@@ -6815,7 +6821,7 @@
       <c r="A428" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B428" s="5" t="s">
+      <c r="B428" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C428" s="3"/>
@@ -6824,7 +6830,7 @@
       <c r="A429" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="B429" s="5" t="s">
+      <c r="B429" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C429" s="3"/>
@@ -6833,7 +6839,7 @@
       <c r="A430" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="B430" s="5" t="s">
+      <c r="B430" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C430" s="3"/>
@@ -6842,7 +6848,7 @@
       <c r="A431" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="B431" s="5" t="s">
+      <c r="B431" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C431" s="3"/>
@@ -6851,7 +6857,7 @@
       <c r="A432" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="B432" s="5" t="s">
+      <c r="B432" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C432" s="3"/>
@@ -6860,7 +6866,7 @@
       <c r="A433" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="B433" s="5" t="s">
+      <c r="B433" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C433" s="3"/>
@@ -6869,7 +6875,7 @@
       <c r="A434" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="B434" s="5" t="s">
+      <c r="B434" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C434" s="3"/>
@@ -6878,7 +6884,7 @@
       <c r="A435" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="B435" s="5" t="s">
+      <c r="B435" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C435" s="3"/>
@@ -6887,7 +6893,7 @@
       <c r="A436" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B436" s="5" t="s">
+      <c r="B436" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C436" s="3"/>
@@ -6896,7 +6902,7 @@
       <c r="A437" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="B437" s="5" t="s">
+      <c r="B437" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C437" s="3"/>
@@ -6905,7 +6911,7 @@
       <c r="A438" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="B438" s="5" t="s">
+      <c r="B438" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C438" s="3"/>
@@ -6914,7 +6920,7 @@
       <c r="A439" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="B439" s="5" t="s">
+      <c r="B439" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C439" s="3"/>
@@ -6923,7 +6929,7 @@
       <c r="A440" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="B440" s="5" t="s">
+      <c r="B440" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C440" s="3"/>
@@ -6932,7 +6938,7 @@
       <c r="A441" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="B441" s="5" t="s">
+      <c r="B441" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C441" s="3"/>
@@ -6941,7 +6947,7 @@
       <c r="A442" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B442" s="5" t="s">
+      <c r="B442" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C442" s="3"/>
@@ -6950,7 +6956,7 @@
       <c r="A443" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="B443" s="5" t="s">
+      <c r="B443" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C443" s="3"/>
@@ -6959,7 +6965,7 @@
       <c r="A444" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="B444" s="5" t="s">
+      <c r="B444" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C444" s="3"/>
@@ -6968,7 +6974,7 @@
       <c r="A445" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="B445" s="5" t="s">
+      <c r="B445" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C445" s="3"/>
@@ -6977,7 +6983,7 @@
       <c r="A446" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B446" s="5" t="s">
+      <c r="B446" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C446" s="3"/>
@@ -6986,7 +6992,7 @@
       <c r="A447" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="B447" s="5" t="s">
+      <c r="B447" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C447" s="3"/>
@@ -6995,7 +7001,7 @@
       <c r="A448" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B448" s="5" t="s">
+      <c r="B448" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C448" s="3"/>
@@ -7004,7 +7010,7 @@
       <c r="A449" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="B449" s="5" t="s">
+      <c r="B449" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C449" s="3"/>
@@ -7013,7 +7019,7 @@
       <c r="A450" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B450" s="5" t="s">
+      <c r="B450" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C450" s="3"/>
@@ -7022,7 +7028,7 @@
       <c r="A451" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="B451" s="5" t="s">
+      <c r="B451" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C451" s="3"/>
@@ -7031,7 +7037,7 @@
       <c r="A452" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B452" s="5" t="s">
+      <c r="B452" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C452" s="3"/>
@@ -7040,7 +7046,7 @@
       <c r="A453" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="B453" s="5" t="s">
+      <c r="B453" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C453" s="3"/>
@@ -7049,7 +7055,7 @@
       <c r="A454" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="B454" s="5" t="s">
+      <c r="B454" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C454" s="3"/>
@@ -7058,7 +7064,7 @@
       <c r="A455" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="B455" s="5" t="s">
+      <c r="B455" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C455" s="3"/>
@@ -7067,7 +7073,7 @@
       <c r="A456" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="B456" s="5" t="s">
+      <c r="B456" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C456" s="3"/>
@@ -7076,7 +7082,7 @@
       <c r="A457" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="B457" s="5" t="s">
+      <c r="B457" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C457" s="3"/>
@@ -7085,7 +7091,7 @@
       <c r="A458" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="B458" s="5" t="s">
+      <c r="B458" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C458" s="3"/>
@@ -7094,7 +7100,7 @@
       <c r="A459" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="B459" s="5" t="s">
+      <c r="B459" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C459" s="3"/>
@@ -7103,7 +7109,7 @@
       <c r="A460" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="B460" s="5" t="s">
+      <c r="B460" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C460" s="3"/>
@@ -7112,7 +7118,7 @@
       <c r="A461" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="B461" s="5" t="s">
+      <c r="B461" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C461" s="3"/>
@@ -7121,7 +7127,7 @@
       <c r="A462" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="B462" s="5" t="s">
+      <c r="B462" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C462" s="3"/>
@@ -7130,7 +7136,7 @@
       <c r="A463" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="B463" s="5" t="s">
+      <c r="B463" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C463" s="3"/>
@@ -7139,7 +7145,7 @@
       <c r="A464" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="B464" s="5" t="s">
+      <c r="B464" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C464" s="3"/>
@@ -7148,7 +7154,7 @@
       <c r="A465" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="B465" s="5" t="s">
+      <c r="B465" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C465" s="3"/>
@@ -7157,7 +7163,7 @@
       <c r="A466" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="B466" s="5" t="s">
+      <c r="B466" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C466" s="3"/>
@@ -7166,7 +7172,7 @@
       <c r="A467" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="B467" s="5" t="s">
+      <c r="B467" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C467" s="3"/>
@@ -7175,7 +7181,7 @@
       <c r="A468" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="B468" s="5" t="s">
+      <c r="B468" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C468" s="3"/>
@@ -7184,7 +7190,7 @@
       <c r="A469" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="B469" s="5" t="s">
+      <c r="B469" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C469" s="3"/>
@@ -7193,7 +7199,7 @@
       <c r="A470" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="B470" s="5" t="s">
+      <c r="B470" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C470" s="3"/>
@@ -7202,7 +7208,7 @@
       <c r="A471" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="B471" s="5" t="s">
+      <c r="B471" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C471" s="3"/>
@@ -7211,7 +7217,7 @@
       <c r="A472" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="B472" s="5" t="s">
+      <c r="B472" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C472" s="3"/>
@@ -7220,7 +7226,7 @@
       <c r="A473" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="B473" s="5" t="s">
+      <c r="B473" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C473" s="3"/>
@@ -7229,7 +7235,7 @@
       <c r="A474" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="B474" s="5" t="s">
+      <c r="B474" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C474" s="3"/>
@@ -7238,7 +7244,7 @@
       <c r="A475" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="B475" s="5" t="s">
+      <c r="B475" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C475" s="3"/>
@@ -7247,7 +7253,7 @@
       <c r="A476" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="B476" s="5" t="s">
+      <c r="B476" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C476" s="3"/>
@@ -7256,7 +7262,7 @@
       <c r="A477" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="B477" s="5" t="s">
+      <c r="B477" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C477" s="3"/>
@@ -7265,7 +7271,7 @@
       <c r="A478" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="B478" s="5" t="s">
+      <c r="B478" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C478" s="3"/>
@@ -7274,7 +7280,7 @@
       <c r="A479" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="B479" s="5" t="s">
+      <c r="B479" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C479" s="3"/>
@@ -7283,7 +7289,7 @@
       <c r="A480" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="B480" s="5" t="s">
+      <c r="B480" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C480" s="3"/>
@@ -7292,7 +7298,7 @@
       <c r="A481" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="B481" s="5" t="s">
+      <c r="B481" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C481" s="3"/>
@@ -7301,7 +7307,7 @@
       <c r="A482" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="B482" s="5" t="s">
+      <c r="B482" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C482" s="3"/>
@@ -7310,7 +7316,7 @@
       <c r="A483" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="B483" s="5" t="s">
+      <c r="B483" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C483" s="3"/>
@@ -7319,7 +7325,7 @@
       <c r="A484" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="B484" s="5" t="s">
+      <c r="B484" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C484" s="3"/>
@@ -7328,7 +7334,7 @@
       <c r="A485" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="B485" s="5" t="s">
+      <c r="B485" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C485" s="3"/>
@@ -7337,7 +7343,7 @@
       <c r="A486" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="B486" s="5" t="s">
+      <c r="B486" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C486" s="3"/>
@@ -7346,7 +7352,7 @@
       <c r="A487" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="B487" s="5" t="s">
+      <c r="B487" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C487" s="3"/>
@@ -7355,7 +7361,7 @@
       <c r="A488" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="B488" s="5" t="s">
+      <c r="B488" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C488" s="3"/>
@@ -7364,7 +7370,7 @@
       <c r="A489" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="B489" s="5" t="s">
+      <c r="B489" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C489" s="3"/>
@@ -7373,7 +7379,7 @@
       <c r="A490" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="B490" s="5" t="s">
+      <c r="B490" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C490" s="3"/>
@@ -7382,7 +7388,7 @@
       <c r="A491" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="B491" s="5" t="s">
+      <c r="B491" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C491" s="3"/>
@@ -7391,7 +7397,7 @@
       <c r="A492" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="B492" s="5" t="s">
+      <c r="B492" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C492" s="3"/>
@@ -7400,7 +7406,7 @@
       <c r="A493" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="B493" s="5" t="s">
+      <c r="B493" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C493" s="3"/>
@@ -7409,7 +7415,7 @@
       <c r="A494" s="1" t="s">
         <v>496</v>
       </c>
-      <c r="B494" s="5" t="s">
+      <c r="B494" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C494" s="3"/>
@@ -7418,7 +7424,7 @@
       <c r="A495" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="B495" s="5" t="s">
+      <c r="B495" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C495" s="3"/>
@@ -7427,7 +7433,7 @@
       <c r="A496" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="B496" s="5" t="s">
+      <c r="B496" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C496" s="3"/>
@@ -7436,7 +7442,7 @@
       <c r="A497" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="B497" s="5" t="s">
+      <c r="B497" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C497" s="3"/>
@@ -7445,7 +7451,7 @@
       <c r="A498" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="B498" s="5" t="s">
+      <c r="B498" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C498" s="3"/>
@@ -7454,7 +7460,7 @@
       <c r="A499" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="B499" s="5" t="s">
+      <c r="B499" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C499" s="3"/>
@@ -7463,7 +7469,7 @@
       <c r="A500" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="B500" s="5" t="s">
+      <c r="B500" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C500" s="3"/>
@@ -7472,7 +7478,7 @@
       <c r="A501" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="B501" s="5" t="s">
+      <c r="B501" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C501" s="3"/>
@@ -7481,7 +7487,7 @@
       <c r="A502" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="B502" s="5" t="s">
+      <c r="B502" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C502" s="3"/>
@@ -7490,7 +7496,7 @@
       <c r="A503" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="B503" s="5" t="s">
+      <c r="B503" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C503" s="3"/>
@@ -7499,7 +7505,7 @@
       <c r="A504" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="B504" s="5" t="s">
+      <c r="B504" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C504" s="3"/>
@@ -7508,7 +7514,7 @@
       <c r="A505" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="B505" s="5" t="s">
+      <c r="B505" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C505" s="3"/>
@@ -7517,7 +7523,7 @@
       <c r="A506" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="B506" s="5" t="s">
+      <c r="B506" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C506" s="3"/>
@@ -7526,7 +7532,7 @@
       <c r="A507" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="B507" s="5" t="s">
+      <c r="B507" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C507" s="3"/>
@@ -7535,7 +7541,7 @@
       <c r="A508" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="B508" s="5" t="s">
+      <c r="B508" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C508" s="3"/>
@@ -7544,7 +7550,7 @@
       <c r="A509" s="1" t="s">
         <v>511</v>
       </c>
-      <c r="B509" s="5" t="s">
+      <c r="B509" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C509" s="3"/>
@@ -7553,7 +7559,7 @@
       <c r="A510" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="B510" s="5" t="s">
+      <c r="B510" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C510" s="3"/>
@@ -7562,7 +7568,7 @@
       <c r="A511" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="B511" s="5" t="s">
+      <c r="B511" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C511" s="3"/>
@@ -7571,7 +7577,7 @@
       <c r="A512" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="B512" s="5" t="s">
+      <c r="B512" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C512" s="3"/>
@@ -7580,7 +7586,7 @@
       <c r="A513" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="B513" s="5" t="s">
+      <c r="B513" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C513" s="3"/>
@@ -7589,7 +7595,7 @@
       <c r="A514" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="B514" s="5" t="s">
+      <c r="B514" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C514" s="3"/>
@@ -7598,7 +7604,7 @@
       <c r="A515" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="B515" s="5" t="s">
+      <c r="B515" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C515" s="3"/>
@@ -7607,7 +7613,7 @@
       <c r="A516" s="1" t="s">
         <v>518</v>
       </c>
-      <c r="B516" s="5" t="s">
+      <c r="B516" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C516" s="3"/>
@@ -7616,7 +7622,7 @@
       <c r="A517" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="B517" s="5" t="s">
+      <c r="B517" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C517" s="3"/>
@@ -7625,7 +7631,7 @@
       <c r="A518" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="B518" s="5" t="s">
+      <c r="B518" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C518" s="3"/>
@@ -7634,7 +7640,7 @@
       <c r="A519" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="B519" s="5" t="s">
+      <c r="B519" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C519" s="3"/>
@@ -7643,7 +7649,7 @@
       <c r="A520" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="B520" s="5" t="s">
+      <c r="B520" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C520" s="3"/>
@@ -7652,7 +7658,7 @@
       <c r="A521" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="B521" s="5" t="s">
+      <c r="B521" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C521" s="3"/>
@@ -7661,7 +7667,7 @@
       <c r="A522" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="B522" s="5" t="s">
+      <c r="B522" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C522" s="3"/>
@@ -7670,7 +7676,7 @@
       <c r="A523" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="B523" s="5" t="s">
+      <c r="B523" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C523" s="3"/>
@@ -7679,7 +7685,7 @@
       <c r="A524" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="B524" s="5" t="s">
+      <c r="B524" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C524" s="3"/>
@@ -7688,7 +7694,7 @@
       <c r="A525" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="B525" s="5" t="s">
+      <c r="B525" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C525" s="3"/>
@@ -7697,7 +7703,7 @@
       <c r="A526" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="B526" s="5" t="s">
+      <c r="B526" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C526" s="3"/>
@@ -7706,7 +7712,7 @@
       <c r="A527" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="B527" s="5" t="s">
+      <c r="B527" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C527" s="3"/>
@@ -7715,7 +7721,7 @@
       <c r="A528" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="B528" s="5" t="s">
+      <c r="B528" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C528" s="3"/>
@@ -7724,7 +7730,7 @@
       <c r="A529" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="B529" s="5" t="s">
+      <c r="B529" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C529" s="3"/>
@@ -7733,7 +7739,7 @@
       <c r="A530" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="B530" s="5" t="s">
+      <c r="B530" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C530" s="3"/>
@@ -7742,7 +7748,7 @@
       <c r="A531" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="B531" s="5" t="s">
+      <c r="B531" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C531" s="3"/>
@@ -7751,7 +7757,7 @@
       <c r="A532" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="B532" s="5" t="s">
+      <c r="B532" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C532" s="3"/>
@@ -7760,7 +7766,7 @@
       <c r="A533" s="1" t="s">
         <v>535</v>
       </c>
-      <c r="B533" s="5" t="s">
+      <c r="B533" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C533" s="3"/>
@@ -7769,7 +7775,7 @@
       <c r="A534" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="B534" s="5" t="s">
+      <c r="B534" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C534" s="3"/>
@@ -7778,7 +7784,7 @@
       <c r="A535" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="B535" s="5" t="s">
+      <c r="B535" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C535" s="3"/>
@@ -7787,7 +7793,7 @@
       <c r="A536" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="B536" s="5" t="s">
+      <c r="B536" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C536" s="3"/>
@@ -7796,7 +7802,7 @@
       <c r="A537" s="1" t="s">
         <v>539</v>
       </c>
-      <c r="B537" s="5" t="s">
+      <c r="B537" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C537" s="3"/>
@@ -7805,7 +7811,7 @@
       <c r="A538" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="B538" s="5" t="s">
+      <c r="B538" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C538" s="3"/>
@@ -7814,7 +7820,7 @@
       <c r="A539" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="B539" s="5" t="s">
+      <c r="B539" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C539" s="3"/>
@@ -7823,7 +7829,7 @@
       <c r="A540" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="B540" s="5" t="s">
+      <c r="B540" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C540" s="3"/>
@@ -7832,7 +7838,7 @@
       <c r="A541" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="B541" s="5" t="s">
+      <c r="B541" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C541" s="3"/>
@@ -7841,7 +7847,7 @@
       <c r="A542" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="B542" s="5" t="s">
+      <c r="B542" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C542" s="3"/>
@@ -7850,7 +7856,7 @@
       <c r="A543" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="B543" s="5" t="s">
+      <c r="B543" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C543" s="3"/>
@@ -7859,7 +7865,7 @@
       <c r="A544" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="B544" s="5" t="s">
+      <c r="B544" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C544" s="3"/>
@@ -7868,7 +7874,7 @@
       <c r="A545" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="B545" s="5" t="s">
+      <c r="B545" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C545" s="3"/>
@@ -7877,7 +7883,7 @@
       <c r="A546" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="B546" s="5" t="s">
+      <c r="B546" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C546" s="3"/>
@@ -7886,7 +7892,7 @@
       <c r="A547" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="B547" s="5" t="s">
+      <c r="B547" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C547" s="3"/>
@@ -7895,7 +7901,7 @@
       <c r="A548" s="1" t="s">
         <v>550</v>
       </c>
-      <c r="B548" s="5" t="s">
+      <c r="B548" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C548" s="3"/>
@@ -7904,7 +7910,7 @@
       <c r="A549" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="B549" s="5" t="s">
+      <c r="B549" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C549" s="3"/>
@@ -7913,7 +7919,7 @@
       <c r="A550" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="B550" s="5" t="s">
+      <c r="B550" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C550" s="3"/>
@@ -7922,7 +7928,7 @@
       <c r="A551" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="B551" s="5" t="s">
+      <c r="B551" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C551" s="3"/>
@@ -7931,7 +7937,7 @@
       <c r="A552" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="B552" s="5" t="s">
+      <c r="B552" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C552" s="3"/>
@@ -7940,7 +7946,7 @@
       <c r="A553" s="1" t="s">
         <v>555</v>
       </c>
-      <c r="B553" s="5" t="s">
+      <c r="B553" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C553" s="3"/>
@@ -7949,7 +7955,7 @@
       <c r="A554" s="1" t="s">
         <v>556</v>
       </c>
-      <c r="B554" s="5" t="s">
+      <c r="B554" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C554" s="3"/>
@@ -7958,7 +7964,7 @@
       <c r="A555" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="B555" s="5" t="s">
+      <c r="B555" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C555" s="3"/>
@@ -7967,7 +7973,7 @@
       <c r="A556" s="1" t="s">
         <v>558</v>
       </c>
-      <c r="B556" s="5" t="s">
+      <c r="B556" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C556" s="3"/>
@@ -7976,7 +7982,7 @@
       <c r="A557" s="1" t="s">
         <v>559</v>
       </c>
-      <c r="B557" s="5" t="s">
+      <c r="B557" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C557" s="3"/>
@@ -7985,7 +7991,7 @@
       <c r="A558" s="1" t="s">
         <v>560</v>
       </c>
-      <c r="B558" s="5" t="s">
+      <c r="B558" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C558" s="3"/>
@@ -7994,7 +8000,7 @@
       <c r="A559" s="1" t="s">
         <v>561</v>
       </c>
-      <c r="B559" s="5" t="s">
+      <c r="B559" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C559" s="3"/>
@@ -8003,7 +8009,7 @@
       <c r="A560" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="B560" s="5" t="s">
+      <c r="B560" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C560" s="3"/>
@@ -8012,7 +8018,7 @@
       <c r="A561" s="1" t="s">
         <v>563</v>
       </c>
-      <c r="B561" s="5" t="s">
+      <c r="B561" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C561" s="3"/>
@@ -8021,7 +8027,7 @@
       <c r="A562" s="1" t="s">
         <v>564</v>
       </c>
-      <c r="B562" s="5" t="s">
+      <c r="B562" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C562" s="3"/>
@@ -8030,7 +8036,7 @@
       <c r="A563" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="B563" s="5" t="s">
+      <c r="B563" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C563" s="3"/>
@@ -8039,7 +8045,7 @@
       <c r="A564" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="B564" s="5" t="s">
+      <c r="B564" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C564" s="3"/>
@@ -8048,7 +8054,7 @@
       <c r="A565" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="B565" s="5" t="s">
+      <c r="B565" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C565" s="3"/>
@@ -8057,7 +8063,7 @@
       <c r="A566" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="B566" s="5" t="s">
+      <c r="B566" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C566" s="3"/>
@@ -8066,7 +8072,7 @@
       <c r="A567" s="1" t="s">
         <v>569</v>
       </c>
-      <c r="B567" s="5" t="s">
+      <c r="B567" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C567" s="3"/>
@@ -8075,7 +8081,7 @@
       <c r="A568" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="B568" s="5" t="s">
+      <c r="B568" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C568" s="3"/>
@@ -8084,7 +8090,7 @@
       <c r="A569" s="1" t="s">
         <v>571</v>
       </c>
-      <c r="B569" s="5" t="s">
+      <c r="B569" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C569" s="3"/>
@@ -8093,7 +8099,7 @@
       <c r="A570" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="B570" s="5" t="s">
+      <c r="B570" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C570" s="3"/>
@@ -8102,7 +8108,7 @@
       <c r="A571" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="B571" s="5" t="s">
+      <c r="B571" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C571" s="3"/>
@@ -8111,7 +8117,7 @@
       <c r="A572" s="1" t="s">
         <v>574</v>
       </c>
-      <c r="B572" s="5" t="s">
+      <c r="B572" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C572" s="3"/>
@@ -8120,7 +8126,7 @@
       <c r="A573" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="B573" s="5" t="s">
+      <c r="B573" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C573" s="3"/>
@@ -8129,7 +8135,7 @@
       <c r="A574" s="1" t="s">
         <v>576</v>
       </c>
-      <c r="B574" s="5" t="s">
+      <c r="B574" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C574" s="3"/>
@@ -8138,7 +8144,7 @@
       <c r="A575" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B575" s="5" t="s">
+      <c r="B575" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C575" s="3"/>
@@ -8147,7 +8153,7 @@
       <c r="A576" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="B576" s="5" t="s">
+      <c r="B576" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C576" s="3"/>
@@ -8156,7 +8162,7 @@
       <c r="A577" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="B577" s="5" t="s">
+      <c r="B577" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C577" s="3"/>
@@ -8165,7 +8171,7 @@
       <c r="A578" s="1" t="s">
         <v>580</v>
       </c>
-      <c r="B578" s="5" t="s">
+      <c r="B578" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C578" s="3"/>
@@ -8174,7 +8180,7 @@
       <c r="A579" s="1" t="s">
         <v>581</v>
       </c>
-      <c r="B579" s="5" t="s">
+      <c r="B579" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C579" s="3"/>
@@ -8183,7 +8189,7 @@
       <c r="A580" s="1" t="s">
         <v>582</v>
       </c>
-      <c r="B580" s="5" t="s">
+      <c r="B580" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C580" s="3"/>
@@ -8192,7 +8198,7 @@
       <c r="A581" s="1" t="s">
         <v>583</v>
       </c>
-      <c r="B581" s="5" t="s">
+      <c r="B581" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C581" s="3"/>
@@ -8201,7 +8207,7 @@
       <c r="A582" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="B582" s="5" t="s">
+      <c r="B582" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C582" s="3"/>
@@ -8210,7 +8216,7 @@
       <c r="A583" s="1" t="s">
         <v>585</v>
       </c>
-      <c r="B583" s="5" t="s">
+      <c r="B583" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C583" s="3"/>
@@ -8219,7 +8225,7 @@
       <c r="A584" s="1" t="s">
         <v>586</v>
       </c>
-      <c r="B584" s="5" t="s">
+      <c r="B584" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C584" s="3"/>
@@ -8228,7 +8234,7 @@
       <c r="A585" s="1" t="s">
         <v>587</v>
       </c>
-      <c r="B585" s="5" t="s">
+      <c r="B585" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C585" s="3"/>
@@ -8237,7 +8243,7 @@
       <c r="A586" s="1" t="s">
         <v>588</v>
       </c>
-      <c r="B586" s="5" t="s">
+      <c r="B586" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C586" s="3"/>
@@ -8246,7 +8252,7 @@
       <c r="A587" s="1" t="s">
         <v>589</v>
       </c>
-      <c r="B587" s="5" t="s">
+      <c r="B587" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C587" s="3"/>
@@ -8255,7 +8261,7 @@
       <c r="A588" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="B588" s="5" t="s">
+      <c r="B588" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C588" s="3"/>
@@ -8264,7 +8270,7 @@
       <c r="A589" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="B589" s="5" t="s">
+      <c r="B589" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C589" s="3"/>
@@ -8273,7 +8279,7 @@
       <c r="A590" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="B590" s="5" t="s">
+      <c r="B590" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C590" s="3"/>
@@ -8282,7 +8288,7 @@
       <c r="A591" s="1" t="s">
         <v>593</v>
       </c>
-      <c r="B591" s="5" t="s">
+      <c r="B591" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C591" s="3"/>
@@ -8291,7 +8297,7 @@
       <c r="A592" s="1" t="s">
         <v>594</v>
       </c>
-      <c r="B592" s="5" t="s">
+      <c r="B592" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C592" s="3"/>
@@ -8300,7 +8306,7 @@
       <c r="A593" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="B593" s="5" t="s">
+      <c r="B593" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C593" s="3"/>
@@ -8309,7 +8315,7 @@
       <c r="A594" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="B594" s="5" t="s">
+      <c r="B594" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C594" s="3"/>
@@ -8318,7 +8324,7 @@
       <c r="A595" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="B595" s="5" t="s">
+      <c r="B595" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C595" s="3"/>
@@ -8327,7 +8333,7 @@
       <c r="A596" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="B596" s="5" t="s">
+      <c r="B596" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C596" s="3"/>
@@ -8336,7 +8342,7 @@
       <c r="A597" s="1" t="s">
         <v>599</v>
       </c>
-      <c r="B597" s="5" t="s">
+      <c r="B597" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C597" s="3"/>
@@ -8345,7 +8351,7 @@
       <c r="A598" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="B598" s="5" t="s">
+      <c r="B598" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C598" s="3"/>
@@ -8354,7 +8360,7 @@
       <c r="A599" s="1" t="s">
         <v>601</v>
       </c>
-      <c r="B599" s="5" t="s">
+      <c r="B599" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C599" s="3"/>
@@ -8363,7 +8369,7 @@
       <c r="A600" s="1" t="s">
         <v>602</v>
       </c>
-      <c r="B600" s="5" t="s">
+      <c r="B600" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C600" s="3"/>
@@ -8372,7 +8378,7 @@
       <c r="A601" s="1" t="s">
         <v>603</v>
       </c>
-      <c r="B601" s="5" t="s">
+      <c r="B601" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C601" s="3"/>
@@ -8381,7 +8387,7 @@
       <c r="A602" s="1" t="s">
         <v>604</v>
       </c>
-      <c r="B602" s="5" t="s">
+      <c r="B602" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C602" s="3"/>
@@ -8390,7 +8396,7 @@
       <c r="A603" s="1" t="s">
         <v>605</v>
       </c>
-      <c r="B603" s="5" t="s">
+      <c r="B603" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C603" s="3"/>
@@ -8399,7 +8405,7 @@
       <c r="A604" s="1" t="s">
         <v>606</v>
       </c>
-      <c r="B604" s="5" t="s">
+      <c r="B604" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C604" s="3"/>
@@ -8408,7 +8414,7 @@
       <c r="A605" s="1" t="s">
         <v>607</v>
       </c>
-      <c r="B605" s="5" t="s">
+      <c r="B605" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C605" s="3"/>
@@ -8417,7 +8423,7 @@
       <c r="A606" s="1" t="s">
         <v>608</v>
       </c>
-      <c r="B606" s="5" t="s">
+      <c r="B606" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C606" s="3"/>
@@ -8426,7 +8432,7 @@
       <c r="A607" s="1" t="s">
         <v>609</v>
       </c>
-      <c r="B607" s="5" t="s">
+      <c r="B607" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C607" s="3"/>
@@ -8435,7 +8441,7 @@
       <c r="A608" s="1" t="s">
         <v>610</v>
       </c>
-      <c r="B608" s="5" t="s">
+      <c r="B608" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C608" s="3"/>
@@ -8444,7 +8450,7 @@
       <c r="A609" s="1" t="s">
         <v>611</v>
       </c>
-      <c r="B609" s="5" t="s">
+      <c r="B609" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C609" s="3"/>
@@ -8453,7 +8459,7 @@
       <c r="A610" s="1" t="s">
         <v>612</v>
       </c>
-      <c r="B610" s="5" t="s">
+      <c r="B610" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C610" s="3"/>
@@ -8462,7 +8468,7 @@
       <c r="A611" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="B611" s="5" t="s">
+      <c r="B611" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C611" s="3"/>
@@ -8471,7 +8477,7 @@
       <c r="A612" s="1" t="s">
         <v>614</v>
       </c>
-      <c r="B612" s="5" t="s">
+      <c r="B612" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C612" s="3"/>
@@ -8480,7 +8486,7 @@
       <c r="A613" s="1" t="s">
         <v>615</v>
       </c>
-      <c r="B613" s="5" t="s">
+      <c r="B613" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C613" s="3"/>
@@ -8489,7 +8495,7 @@
       <c r="A614" s="1" t="s">
         <v>616</v>
       </c>
-      <c r="B614" s="5" t="s">
+      <c r="B614" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C614" s="3"/>
@@ -8498,7 +8504,7 @@
       <c r="A615" s="1" t="s">
         <v>617</v>
       </c>
-      <c r="B615" s="5" t="s">
+      <c r="B615" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C615" s="3"/>
@@ -8507,7 +8513,7 @@
       <c r="A616" s="1" t="s">
         <v>618</v>
       </c>
-      <c r="B616" s="5" t="s">
+      <c r="B616" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C616" s="3"/>
@@ -8516,7 +8522,7 @@
       <c r="A617" s="1" t="s">
         <v>619</v>
       </c>
-      <c r="B617" s="5" t="s">
+      <c r="B617" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C617" s="3"/>
@@ -8525,7 +8531,7 @@
       <c r="A618" s="1" t="s">
         <v>620</v>
       </c>
-      <c r="B618" s="5" t="s">
+      <c r="B618" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C618" s="3"/>
@@ -8534,7 +8540,7 @@
       <c r="A619" s="1" t="s">
         <v>621</v>
       </c>
-      <c r="B619" s="5" t="s">
+      <c r="B619" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C619" s="3"/>
@@ -8543,7 +8549,7 @@
       <c r="A620" s="1" t="s">
         <v>622</v>
       </c>
-      <c r="B620" s="5" t="s">
+      <c r="B620" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C620" s="3"/>
@@ -8552,7 +8558,7 @@
       <c r="A621" s="1" t="s">
         <v>623</v>
       </c>
-      <c r="B621" s="5" t="s">
+      <c r="B621" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C621" s="3"/>
@@ -8561,7 +8567,7 @@
       <c r="A622" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="B622" s="5" t="s">
+      <c r="B622" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C622" s="3"/>
@@ -8570,7 +8576,7 @@
       <c r="A623" s="1" t="s">
         <v>625</v>
       </c>
-      <c r="B623" s="5" t="s">
+      <c r="B623" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C623" s="3"/>
@@ -8579,7 +8585,7 @@
       <c r="A624" s="1" t="s">
         <v>626</v>
       </c>
-      <c r="B624" s="5" t="s">
+      <c r="B624" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C624" s="3"/>
@@ -8588,7 +8594,7 @@
       <c r="A625" s="1" t="s">
         <v>627</v>
       </c>
-      <c r="B625" s="5" t="s">
+      <c r="B625" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C625" s="3"/>
@@ -8597,7 +8603,7 @@
       <c r="A626" s="1" t="s">
         <v>628</v>
       </c>
-      <c r="B626" s="5" t="s">
+      <c r="B626" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C626" s="3"/>
@@ -8606,7 +8612,7 @@
       <c r="A627" s="1" t="s">
         <v>629</v>
       </c>
-      <c r="B627" s="5" t="s">
+      <c r="B627" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C627" s="3"/>
@@ -8615,7 +8621,7 @@
       <c r="A628" s="1" t="s">
         <v>630</v>
       </c>
-      <c r="B628" s="5" t="s">
+      <c r="B628" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C628" s="3"/>
@@ -8624,7 +8630,7 @@
       <c r="A629" s="1" t="s">
         <v>631</v>
       </c>
-      <c r="B629" s="5" t="s">
+      <c r="B629" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C629" s="3"/>
@@ -8633,7 +8639,7 @@
       <c r="A630" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="B630" s="5" t="s">
+      <c r="B630" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C630" s="3"/>
@@ -8642,7 +8648,7 @@
       <c r="A631" s="1" t="s">
         <v>633</v>
       </c>
-      <c r="B631" s="5" t="s">
+      <c r="B631" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C631" s="3"/>
@@ -8651,7 +8657,7 @@
       <c r="A632" s="1" t="s">
         <v>634</v>
       </c>
-      <c r="B632" s="5" t="s">
+      <c r="B632" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C632" s="3"/>
@@ -8660,7 +8666,7 @@
       <c r="A633" s="1" t="s">
         <v>635</v>
       </c>
-      <c r="B633" s="5" t="s">
+      <c r="B633" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C633" s="3"/>
@@ -8669,7 +8675,7 @@
       <c r="A634" s="1" t="s">
         <v>636</v>
       </c>
-      <c r="B634" s="5" t="s">
+      <c r="B634" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C634" s="3"/>
@@ -8678,7 +8684,7 @@
       <c r="A635" s="1" t="s">
         <v>637</v>
       </c>
-      <c r="B635" s="5" t="s">
+      <c r="B635" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C635" s="3"/>
@@ -8687,7 +8693,7 @@
       <c r="A636" s="1" t="s">
         <v>638</v>
       </c>
-      <c r="B636" s="5" t="s">
+      <c r="B636" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C636" s="3"/>
@@ -8696,7 +8702,7 @@
       <c r="A637" s="1" t="s">
         <v>639</v>
       </c>
-      <c r="B637" s="5" t="s">
+      <c r="B637" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C637" s="3"/>
@@ -8705,7 +8711,7 @@
       <c r="A638" s="1" t="s">
         <v>640</v>
       </c>
-      <c r="B638" s="5" t="s">
+      <c r="B638" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C638" s="3"/>
@@ -8714,7 +8720,7 @@
       <c r="A639" s="1" t="s">
         <v>641</v>
       </c>
-      <c r="B639" s="5" t="s">
+      <c r="B639" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C639" s="3"/>
@@ -8723,7 +8729,7 @@
       <c r="A640" s="1" t="s">
         <v>642</v>
       </c>
-      <c r="B640" s="5" t="s">
+      <c r="B640" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C640" s="3"/>
@@ -8732,7 +8738,7 @@
       <c r="A641" s="1" t="s">
         <v>643</v>
       </c>
-      <c r="B641" s="5" t="s">
+      <c r="B641" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C641" s="3"/>
@@ -8741,7 +8747,7 @@
       <c r="A642" s="1" t="s">
         <v>644</v>
       </c>
-      <c r="B642" s="5" t="s">
+      <c r="B642" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C642" s="3"/>
@@ -8750,7 +8756,7 @@
       <c r="A643" s="1" t="s">
         <v>645</v>
       </c>
-      <c r="B643" s="5" t="s">
+      <c r="B643" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C643" s="3"/>
@@ -8759,7 +8765,7 @@
       <c r="A644" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="B644" s="5" t="s">
+      <c r="B644" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C644" s="3"/>
@@ -8768,7 +8774,7 @@
       <c r="A645" s="1" t="s">
         <v>647</v>
       </c>
-      <c r="B645" s="5" t="s">
+      <c r="B645" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C645" s="3"/>
@@ -8777,7 +8783,7 @@
       <c r="A646" s="1" t="s">
         <v>648</v>
       </c>
-      <c r="B646" s="5" t="s">
+      <c r="B646" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C646" s="3"/>
@@ -8786,7 +8792,7 @@
       <c r="A647" s="1" t="s">
         <v>649</v>
       </c>
-      <c r="B647" s="5" t="s">
+      <c r="B647" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C647" s="3"/>
@@ -8795,7 +8801,7 @@
       <c r="A648" s="1" t="s">
         <v>650</v>
       </c>
-      <c r="B648" s="5" t="s">
+      <c r="B648" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C648" s="3"/>
@@ -8804,7 +8810,7 @@
       <c r="A649" s="1" t="s">
         <v>651</v>
       </c>
-      <c r="B649" s="5" t="s">
+      <c r="B649" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C649" s="3"/>
@@ -8813,7 +8819,7 @@
       <c r="A650" s="1" t="s">
         <v>652</v>
       </c>
-      <c r="B650" s="5" t="s">
+      <c r="B650" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C650" s="3"/>
@@ -8822,7 +8828,7 @@
       <c r="A651" s="1" t="s">
         <v>653</v>
       </c>
-      <c r="B651" s="5" t="s">
+      <c r="B651" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C651" s="3"/>
@@ -8831,7 +8837,7 @@
       <c r="A652" s="1" t="s">
         <v>654</v>
       </c>
-      <c r="B652" s="5" t="s">
+      <c r="B652" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C652" s="3"/>
@@ -8840,7 +8846,7 @@
       <c r="A653" s="1" t="s">
         <v>655</v>
       </c>
-      <c r="B653" s="5" t="s">
+      <c r="B653" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C653" s="3"/>
@@ -8849,7 +8855,7 @@
       <c r="A654" s="1" t="s">
         <v>656</v>
       </c>
-      <c r="B654" s="5" t="s">
+      <c r="B654" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C654" s="3"/>
@@ -8858,7 +8864,7 @@
       <c r="A655" s="1" t="s">
         <v>657</v>
       </c>
-      <c r="B655" s="5" t="s">
+      <c r="B655" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C655" s="3"/>
@@ -8867,7 +8873,7 @@
       <c r="A656" s="1" t="s">
         <v>658</v>
       </c>
-      <c r="B656" s="5" t="s">
+      <c r="B656" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C656" s="3"/>
@@ -8876,7 +8882,7 @@
       <c r="A657" s="1" t="s">
         <v>659</v>
       </c>
-      <c r="B657" s="5" t="s">
+      <c r="B657" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C657" s="3"/>
@@ -8885,7 +8891,7 @@
       <c r="A658" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="B658" s="5" t="s">
+      <c r="B658" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C658" s="3"/>
@@ -8894,7 +8900,7 @@
       <c r="A659" s="1" t="s">
         <v>661</v>
       </c>
-      <c r="B659" s="5" t="s">
+      <c r="B659" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C659" s="3"/>
@@ -8903,7 +8909,7 @@
       <c r="A660" s="1" t="s">
         <v>662</v>
       </c>
-      <c r="B660" s="5" t="s">
+      <c r="B660" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C660" s="3"/>
@@ -8912,7 +8918,7 @@
       <c r="A661" s="1" t="s">
         <v>663</v>
       </c>
-      <c r="B661" s="5" t="s">
+      <c r="B661" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C661" s="3"/>
@@ -8921,7 +8927,7 @@
       <c r="A662" s="1" t="s">
         <v>664</v>
       </c>
-      <c r="B662" s="5" t="s">
+      <c r="B662" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C662" s="3"/>
@@ -8930,7 +8936,7 @@
       <c r="A663" s="1" t="s">
         <v>665</v>
       </c>
-      <c r="B663" s="5" t="s">
+      <c r="B663" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C663" s="3"/>
@@ -8939,7 +8945,7 @@
       <c r="A664" s="1" t="s">
         <v>666</v>
       </c>
-      <c r="B664" s="5" t="s">
+      <c r="B664" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C664" s="3"/>
@@ -8948,7 +8954,7 @@
       <c r="A665" s="1" t="s">
         <v>667</v>
       </c>
-      <c r="B665" s="5" t="s">
+      <c r="B665" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C665" s="3"/>
@@ -8957,7 +8963,7 @@
       <c r="A666" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="B666" s="5" t="s">
+      <c r="B666" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C666" s="3"/>
@@ -8966,7 +8972,7 @@
       <c r="A667" s="1" t="s">
         <v>669</v>
       </c>
-      <c r="B667" s="5" t="s">
+      <c r="B667" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C667" s="3"/>
@@ -8975,7 +8981,7 @@
       <c r="A668" s="1" t="s">
         <v>670</v>
       </c>
-      <c r="B668" s="5" t="s">
+      <c r="B668" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C668" s="3"/>
@@ -8984,7 +8990,7 @@
       <c r="A669" s="1" t="s">
         <v>671</v>
       </c>
-      <c r="B669" s="5" t="s">
+      <c r="B669" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C669" s="3"/>
@@ -8993,7 +8999,7 @@
       <c r="A670" s="1" t="s">
         <v>672</v>
       </c>
-      <c r="B670" s="5" t="s">
+      <c r="B670" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C670" s="3"/>
@@ -9002,7 +9008,7 @@
       <c r="A671" s="1" t="s">
         <v>673</v>
       </c>
-      <c r="B671" s="5" t="s">
+      <c r="B671" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C671" s="3"/>
@@ -9011,7 +9017,7 @@
       <c r="A672" s="1" t="s">
         <v>674</v>
       </c>
-      <c r="B672" s="5" t="s">
+      <c r="B672" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C672" s="3"/>
@@ -9020,7 +9026,7 @@
       <c r="A673" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="B673" s="5" t="s">
+      <c r="B673" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C673" s="3"/>
@@ -9029,7 +9035,7 @@
       <c r="A674" s="1" t="s">
         <v>676</v>
       </c>
-      <c r="B674" s="5" t="s">
+      <c r="B674" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C674" s="3"/>
@@ -9038,7 +9044,7 @@
       <c r="A675" s="1" t="s">
         <v>677</v>
       </c>
-      <c r="B675" s="5" t="s">
+      <c r="B675" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C675" s="3"/>
@@ -9047,7 +9053,7 @@
       <c r="A676" s="1" t="s">
         <v>678</v>
       </c>
-      <c r="B676" s="5" t="s">
+      <c r="B676" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C676" s="3"/>
@@ -9056,7 +9062,7 @@
       <c r="A677" s="1" t="s">
         <v>679</v>
       </c>
-      <c r="B677" s="5" t="s">
+      <c r="B677" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C677" s="3"/>
@@ -9065,7 +9071,7 @@
       <c r="A678" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="B678" s="5" t="s">
+      <c r="B678" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C678" s="3"/>
@@ -9074,7 +9080,7 @@
       <c r="A679" s="1" t="s">
         <v>681</v>
       </c>
-      <c r="B679" s="5" t="s">
+      <c r="B679" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C679" s="3"/>
@@ -9083,7 +9089,7 @@
       <c r="A680" s="1" t="s">
         <v>682</v>
       </c>
-      <c r="B680" s="5" t="s">
+      <c r="B680" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C680" s="3"/>
@@ -9092,7 +9098,7 @@
       <c r="A681" s="1" t="s">
         <v>683</v>
       </c>
-      <c r="B681" s="5" t="s">
+      <c r="B681" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C681" s="3"/>
@@ -9101,7 +9107,7 @@
       <c r="A682" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="B682" s="5" t="s">
+      <c r="B682" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C682" s="3"/>
@@ -9110,7 +9116,7 @@
       <c r="A683" s="1" t="s">
         <v>685</v>
       </c>
-      <c r="B683" s="5" t="s">
+      <c r="B683" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C683" s="3"/>
@@ -9119,7 +9125,7 @@
       <c r="A684" s="1" t="s">
         <v>686</v>
       </c>
-      <c r="B684" s="5" t="s">
+      <c r="B684" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C684" s="3"/>
@@ -9128,7 +9134,7 @@
       <c r="A685" s="1" t="s">
         <v>687</v>
       </c>
-      <c r="B685" s="5" t="s">
+      <c r="B685" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C685" s="3"/>
@@ -9137,7 +9143,7 @@
       <c r="A686" s="1" t="s">
         <v>688</v>
       </c>
-      <c r="B686" s="5" t="s">
+      <c r="B686" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C686" s="3"/>
@@ -9146,7 +9152,7 @@
       <c r="A687" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="B687" s="5" t="s">
+      <c r="B687" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C687" s="3"/>
@@ -9155,7 +9161,7 @@
       <c r="A688" s="1" t="s">
         <v>690</v>
       </c>
-      <c r="B688" s="5" t="s">
+      <c r="B688" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C688" s="3"/>
@@ -9164,7 +9170,7 @@
       <c r="A689" s="1" t="s">
         <v>691</v>
       </c>
-      <c r="B689" s="5" t="s">
+      <c r="B689" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C689" s="3"/>
@@ -9173,7 +9179,7 @@
       <c r="A690" s="1" t="s">
         <v>692</v>
       </c>
-      <c r="B690" s="5" t="s">
+      <c r="B690" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C690" s="3"/>
@@ -9182,7 +9188,7 @@
       <c r="A691" s="1" t="s">
         <v>693</v>
       </c>
-      <c r="B691" s="5" t="s">
+      <c r="B691" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C691" s="3"/>
@@ -9191,7 +9197,7 @@
       <c r="A692" s="1" t="s">
         <v>694</v>
       </c>
-      <c r="B692" s="5" t="s">
+      <c r="B692" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C692" s="3"/>
@@ -9200,7 +9206,7 @@
       <c r="A693" s="1" t="s">
         <v>695</v>
       </c>
-      <c r="B693" s="5" t="s">
+      <c r="B693" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C693" s="3"/>
@@ -9209,7 +9215,7 @@
       <c r="A694" s="1" t="s">
         <v>696</v>
       </c>
-      <c r="B694" s="5" t="s">
+      <c r="B694" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C694" s="3"/>
@@ -9218,7 +9224,7 @@
       <c r="A695" s="1" t="s">
         <v>697</v>
       </c>
-      <c r="B695" s="5" t="s">
+      <c r="B695" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C695" s="3"/>
@@ -9227,7 +9233,7 @@
       <c r="A696" s="1" t="s">
         <v>698</v>
       </c>
-      <c r="B696" s="5" t="s">
+      <c r="B696" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C696" s="3"/>
@@ -9236,7 +9242,7 @@
       <c r="A697" s="1" t="s">
         <v>699</v>
       </c>
-      <c r="B697" s="5" t="s">
+      <c r="B697" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C697" s="3"/>
@@ -9245,7 +9251,7 @@
       <c r="A698" s="1" t="s">
         <v>700</v>
       </c>
-      <c r="B698" s="5" t="s">
+      <c r="B698" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C698" s="3"/>
@@ -9254,7 +9260,7 @@
       <c r="A699" s="1" t="s">
         <v>701</v>
       </c>
-      <c r="B699" s="5" t="s">
+      <c r="B699" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C699" s="3"/>
@@ -9263,7 +9269,7 @@
       <c r="A700" s="1" t="s">
         <v>702</v>
       </c>
-      <c r="B700" s="5" t="s">
+      <c r="B700" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C700" s="3"/>
@@ -9272,7 +9278,7 @@
       <c r="A701" s="1" t="s">
         <v>703</v>
       </c>
-      <c r="B701" s="5" t="s">
+      <c r="B701" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C701" s="3"/>
@@ -9281,7 +9287,7 @@
       <c r="A702" s="1" t="s">
         <v>704</v>
       </c>
-      <c r="B702" s="5" t="s">
+      <c r="B702" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C702" s="3"/>
@@ -9290,7 +9296,7 @@
       <c r="A703" s="1" t="s">
         <v>705</v>
       </c>
-      <c r="B703" s="5" t="s">
+      <c r="B703" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C703" s="3"/>
@@ -9299,7 +9305,7 @@
       <c r="A704" s="1" t="s">
         <v>706</v>
       </c>
-      <c r="B704" s="5" t="s">
+      <c r="B704" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C704" s="3"/>
@@ -9308,7 +9314,7 @@
       <c r="A705" s="1" t="s">
         <v>707</v>
       </c>
-      <c r="B705" s="5" t="s">
+      <c r="B705" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C705" s="3"/>
@@ -9317,7 +9323,7 @@
       <c r="A706" s="1" t="s">
         <v>708</v>
       </c>
-      <c r="B706" s="5" t="s">
+      <c r="B706" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C706" s="3"/>
@@ -9326,7 +9332,7 @@
       <c r="A707" s="1" t="s">
         <v>709</v>
       </c>
-      <c r="B707" s="5" t="s">
+      <c r="B707" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C707" s="3"/>
@@ -9335,7 +9341,7 @@
       <c r="A708" s="1" t="s">
         <v>710</v>
       </c>
-      <c r="B708" s="5" t="s">
+      <c r="B708" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C708" s="3"/>
@@ -9344,7 +9350,7 @@
       <c r="A709" s="1" t="s">
         <v>711</v>
       </c>
-      <c r="B709" s="5" t="s">
+      <c r="B709" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C709" s="3"/>
@@ -9353,7 +9359,7 @@
       <c r="A710" s="1" t="s">
         <v>712</v>
       </c>
-      <c r="B710" s="5" t="s">
+      <c r="B710" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C710" s="3"/>
@@ -9362,7 +9368,7 @@
       <c r="A711" s="1" t="s">
         <v>713</v>
       </c>
-      <c r="B711" s="5" t="s">
+      <c r="B711" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C711" s="3"/>
@@ -9371,7 +9377,7 @@
       <c r="A712" s="1" t="s">
         <v>714</v>
       </c>
-      <c r="B712" s="5" t="s">
+      <c r="B712" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C712" s="3"/>
@@ -9380,7 +9386,7 @@
       <c r="A713" s="1" t="s">
         <v>715</v>
       </c>
-      <c r="B713" s="5" t="s">
+      <c r="B713" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C713" s="3"/>
@@ -9389,7 +9395,7 @@
       <c r="A714" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="B714" s="5" t="s">
+      <c r="B714" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C714" s="3"/>
@@ -9398,7 +9404,7 @@
       <c r="A715" s="1" t="s">
         <v>717</v>
       </c>
-      <c r="B715" s="5" t="s">
+      <c r="B715" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C715" s="3"/>
@@ -9407,7 +9413,7 @@
       <c r="A716" s="1" t="s">
         <v>718</v>
       </c>
-      <c r="B716" s="5" t="s">
+      <c r="B716" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C716" s="3"/>
@@ -9416,7 +9422,7 @@
       <c r="A717" s="1" t="s">
         <v>719</v>
       </c>
-      <c r="B717" s="5" t="s">
+      <c r="B717" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C717" s="3"/>
@@ -9425,7 +9431,7 @@
       <c r="A718" s="1" t="s">
         <v>720</v>
       </c>
-      <c r="B718" s="5" t="s">
+      <c r="B718" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C718" s="3"/>
@@ -9434,7 +9440,7 @@
       <c r="A719" s="1" t="s">
         <v>721</v>
       </c>
-      <c r="B719" s="5" t="s">
+      <c r="B719" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C719" s="3"/>
@@ -9443,7 +9449,7 @@
       <c r="A720" s="1" t="s">
         <v>722</v>
       </c>
-      <c r="B720" s="5" t="s">
+      <c r="B720" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C720" s="3"/>
@@ -9452,7 +9458,7 @@
       <c r="A721" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="B721" s="5" t="s">
+      <c r="B721" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C721" s="3"/>
@@ -9461,7 +9467,7 @@
       <c r="A722" s="1" t="s">
         <v>724</v>
       </c>
-      <c r="B722" s="5" t="s">
+      <c r="B722" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C722" s="3"/>
@@ -9470,7 +9476,7 @@
       <c r="A723" s="1" t="s">
         <v>725</v>
       </c>
-      <c r="B723" s="5" t="s">
+      <c r="B723" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C723" s="3"/>
@@ -9479,7 +9485,7 @@
       <c r="A724" s="1" t="s">
         <v>726</v>
       </c>
-      <c r="B724" s="5" t="s">
+      <c r="B724" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C724" s="3"/>
@@ -9488,7 +9494,7 @@
       <c r="A725" s="1" t="s">
         <v>727</v>
       </c>
-      <c r="B725" s="5" t="s">
+      <c r="B725" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C725" s="3"/>
@@ -9497,7 +9503,7 @@
       <c r="A726" s="1" t="s">
         <v>728</v>
       </c>
-      <c r="B726" s="5" t="s">
+      <c r="B726" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C726" s="3"/>
@@ -9506,7 +9512,7 @@
       <c r="A727" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="B727" s="5" t="s">
+      <c r="B727" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C727" s="3"/>
@@ -9515,7 +9521,7 @@
       <c r="A728" s="1" t="s">
         <v>730</v>
       </c>
-      <c r="B728" s="5" t="s">
+      <c r="B728" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C728" s="3"/>
@@ -9524,7 +9530,7 @@
       <c r="A729" s="1" t="s">
         <v>731</v>
       </c>
-      <c r="B729" s="5" t="s">
+      <c r="B729" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C729" s="3"/>
@@ -9533,7 +9539,7 @@
       <c r="A730" s="1" t="s">
         <v>732</v>
       </c>
-      <c r="B730" s="5" t="s">
+      <c r="B730" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C730" s="3"/>
@@ -9542,7 +9548,7 @@
       <c r="A731" s="1" t="s">
         <v>733</v>
       </c>
-      <c r="B731" s="5" t="s">
+      <c r="B731" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C731" s="3"/>
@@ -9551,7 +9557,7 @@
       <c r="A732" s="1" t="s">
         <v>734</v>
       </c>
-      <c r="B732" s="5" t="s">
+      <c r="B732" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C732" s="3"/>
@@ -9560,7 +9566,7 @@
       <c r="A733" s="1" t="s">
         <v>735</v>
       </c>
-      <c r="B733" s="5" t="s">
+      <c r="B733" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C733" s="3"/>
@@ -9569,7 +9575,7 @@
       <c r="A734" s="1" t="s">
         <v>736</v>
       </c>
-      <c r="B734" s="5" t="s">
+      <c r="B734" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C734" s="3"/>
@@ -9578,7 +9584,7 @@
       <c r="A735" s="1" t="s">
         <v>737</v>
       </c>
-      <c r="B735" s="5" t="s">
+      <c r="B735" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C735" s="3"/>
@@ -9587,7 +9593,7 @@
       <c r="A736" s="1" t="s">
         <v>738</v>
       </c>
-      <c r="B736" s="5" t="s">
+      <c r="B736" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C736" s="3"/>
@@ -9596,7 +9602,7 @@
       <c r="A737" s="1" t="s">
         <v>739</v>
       </c>
-      <c r="B737" s="5" t="s">
+      <c r="B737" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C737" s="3"/>
@@ -9605,7 +9611,7 @@
       <c r="A738" s="1" t="s">
         <v>740</v>
       </c>
-      <c r="B738" s="5" t="s">
+      <c r="B738" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C738" s="3"/>
@@ -9614,7 +9620,7 @@
       <c r="A739" s="1" t="s">
         <v>741</v>
       </c>
-      <c r="B739" s="5" t="s">
+      <c r="B739" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C739" s="3"/>
@@ -9623,7 +9629,7 @@
       <c r="A740" s="1" t="s">
         <v>742</v>
       </c>
-      <c r="B740" s="5" t="s">
+      <c r="B740" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C740" s="3"/>
@@ -9632,7 +9638,7 @@
       <c r="A741" s="1" t="s">
         <v>743</v>
       </c>
-      <c r="B741" s="5" t="s">
+      <c r="B741" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C741" s="3"/>
@@ -9641,7 +9647,7 @@
       <c r="A742" s="1" t="s">
         <v>744</v>
       </c>
-      <c r="B742" s="5" t="s">
+      <c r="B742" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C742" s="3"/>
@@ -9650,7 +9656,7 @@
       <c r="A743" s="1" t="s">
         <v>745</v>
       </c>
-      <c r="B743" s="5" t="s">
+      <c r="B743" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C743" s="3"/>
@@ -9659,7 +9665,7 @@
       <c r="A744" s="1" t="s">
         <v>746</v>
       </c>
-      <c r="B744" s="5" t="s">
+      <c r="B744" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C744" s="3"/>
@@ -9668,7 +9674,7 @@
       <c r="A745" s="1" t="s">
         <v>747</v>
       </c>
-      <c r="B745" s="5" t="s">
+      <c r="B745" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C745" s="3"/>
@@ -9677,7 +9683,7 @@
       <c r="A746" s="1" t="s">
         <v>748</v>
       </c>
-      <c r="B746" s="5" t="s">
+      <c r="B746" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C746" s="3"/>
@@ -9686,7 +9692,7 @@
       <c r="A747" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="B747" s="5" t="s">
+      <c r="B747" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C747" s="3"/>
@@ -9695,7 +9701,7 @@
       <c r="A748" s="1" t="s">
         <v>750</v>
       </c>
-      <c r="B748" s="5" t="s">
+      <c r="B748" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C748" s="3"/>
@@ -9704,7 +9710,7 @@
       <c r="A749" s="1" t="s">
         <v>751</v>
       </c>
-      <c r="B749" s="5" t="s">
+      <c r="B749" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C749" s="3"/>
@@ -9713,7 +9719,7 @@
       <c r="A750" s="1" t="s">
         <v>752</v>
       </c>
-      <c r="B750" s="5" t="s">
+      <c r="B750" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C750" s="3"/>
@@ -9722,7 +9728,7 @@
       <c r="A751" s="1" t="s">
         <v>753</v>
       </c>
-      <c r="B751" s="5" t="s">
+      <c r="B751" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C751" s="3"/>
@@ -9731,7 +9737,7 @@
       <c r="A752" s="1" t="s">
         <v>754</v>
       </c>
-      <c r="B752" s="5" t="s">
+      <c r="B752" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C752" s="3"/>
@@ -9740,7 +9746,7 @@
       <c r="A753" s="1" t="s">
         <v>755</v>
       </c>
-      <c r="B753" s="5" t="s">
+      <c r="B753" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C753" s="3"/>
@@ -9749,7 +9755,7 @@
       <c r="A754" s="1" t="s">
         <v>756</v>
       </c>
-      <c r="B754" s="5" t="s">
+      <c r="B754" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C754" s="3"/>
@@ -9758,7 +9764,7 @@
       <c r="A755" s="1" t="s">
         <v>757</v>
       </c>
-      <c r="B755" s="5" t="s">
+      <c r="B755" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C755" s="3"/>
@@ -9767,7 +9773,7 @@
       <c r="A756" s="1" t="s">
         <v>758</v>
       </c>
-      <c r="B756" s="5" t="s">
+      <c r="B756" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C756" s="3"/>
@@ -9776,7 +9782,7 @@
       <c r="A757" s="1" t="s">
         <v>759</v>
       </c>
-      <c r="B757" s="5" t="s">
+      <c r="B757" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C757" s="3"/>
@@ -9785,7 +9791,7 @@
       <c r="A758" s="1" t="s">
         <v>760</v>
       </c>
-      <c r="B758" s="5" t="s">
+      <c r="B758" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C758" s="3"/>
@@ -9794,7 +9800,7 @@
       <c r="A759" s="1" t="s">
         <v>761</v>
       </c>
-      <c r="B759" s="5" t="s">
+      <c r="B759" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C759" s="3"/>
@@ -9803,7 +9809,7 @@
       <c r="A760" s="1" t="s">
         <v>762</v>
       </c>
-      <c r="B760" s="5" t="s">
+      <c r="B760" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C760" s="3"/>
@@ -9812,7 +9818,7 @@
       <c r="A761" s="1" t="s">
         <v>763</v>
       </c>
-      <c r="B761" s="5" t="s">
+      <c r="B761" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C761" s="3"/>
@@ -9821,7 +9827,7 @@
       <c r="A762" s="1" t="s">
         <v>764</v>
       </c>
-      <c r="B762" s="5" t="s">
+      <c r="B762" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C762" s="3"/>
@@ -9830,7 +9836,7 @@
       <c r="A763" s="1" t="s">
         <v>765</v>
       </c>
-      <c r="B763" s="5" t="s">
+      <c r="B763" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C763" s="3"/>
@@ -9839,7 +9845,7 @@
       <c r="A764" s="1" t="s">
         <v>766</v>
       </c>
-      <c r="B764" s="5" t="s">
+      <c r="B764" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C764" s="3"/>
@@ -9848,7 +9854,7 @@
       <c r="A765" s="1" t="s">
         <v>767</v>
       </c>
-      <c r="B765" s="5" t="s">
+      <c r="B765" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C765" s="3"/>
@@ -9857,7 +9863,7 @@
       <c r="A766" s="1" t="s">
         <v>768</v>
       </c>
-      <c r="B766" s="5" t="s">
+      <c r="B766" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C766" s="3"/>
@@ -9866,7 +9872,7 @@
       <c r="A767" s="1" t="s">
         <v>769</v>
       </c>
-      <c r="B767" s="5" t="s">
+      <c r="B767" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C767" s="3"/>
@@ -9875,7 +9881,7 @@
       <c r="A768" s="1" t="s">
         <v>770</v>
       </c>
-      <c r="B768" s="5" t="s">
+      <c r="B768" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C768" s="3"/>
@@ -9884,7 +9890,7 @@
       <c r="A769" s="1" t="s">
         <v>771</v>
       </c>
-      <c r="B769" s="5" t="s">
+      <c r="B769" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C769" s="3"/>
@@ -9893,7 +9899,7 @@
       <c r="A770" s="1" t="s">
         <v>772</v>
       </c>
-      <c r="B770" s="5" t="s">
+      <c r="B770" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C770" s="3"/>
@@ -9902,7 +9908,7 @@
       <c r="A771" s="1" t="s">
         <v>773</v>
       </c>
-      <c r="B771" s="5" t="s">
+      <c r="B771" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C771" s="3"/>
@@ -9911,7 +9917,7 @@
       <c r="A772" s="1" t="s">
         <v>774</v>
       </c>
-      <c r="B772" s="5" t="s">
+      <c r="B772" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C772" s="3"/>
@@ -9920,7 +9926,7 @@
       <c r="A773" s="1" t="s">
         <v>775</v>
       </c>
-      <c r="B773" s="5" t="s">
+      <c r="B773" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C773" s="3"/>
@@ -9929,7 +9935,7 @@
       <c r="A774" s="1" t="s">
         <v>776</v>
       </c>
-      <c r="B774" s="5" t="s">
+      <c r="B774" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C774" s="3"/>
@@ -9938,7 +9944,7 @@
       <c r="A775" s="1" t="s">
         <v>777</v>
       </c>
-      <c r="B775" s="5" t="s">
+      <c r="B775" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C775" s="3"/>
@@ -9947,7 +9953,7 @@
       <c r="A776" s="1" t="s">
         <v>778</v>
       </c>
-      <c r="B776" s="5" t="s">
+      <c r="B776" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C776" s="3"/>
@@ -9956,7 +9962,7 @@
       <c r="A777" s="1" t="s">
         <v>779</v>
       </c>
-      <c r="B777" s="5" t="s">
+      <c r="B777" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C777" s="3"/>
@@ -9965,7 +9971,7 @@
       <c r="A778" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="B778" s="5" t="s">
+      <c r="B778" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C778" s="3"/>
@@ -9974,7 +9980,7 @@
       <c r="A779" s="1" t="s">
         <v>781</v>
       </c>
-      <c r="B779" s="5" t="s">
+      <c r="B779" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C779" s="3"/>
@@ -9983,7 +9989,7 @@
       <c r="A780" s="1" t="s">
         <v>782</v>
       </c>
-      <c r="B780" s="5" t="s">
+      <c r="B780" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C780" s="3"/>
@@ -9992,7 +9998,7 @@
       <c r="A781" s="1" t="s">
         <v>783</v>
       </c>
-      <c r="B781" s="5" t="s">
+      <c r="B781" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C781" s="3"/>
@@ -10001,7 +10007,7 @@
       <c r="A782" s="1" t="s">
         <v>784</v>
       </c>
-      <c r="B782" s="5" t="s">
+      <c r="B782" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C782" s="3"/>
@@ -10010,7 +10016,7 @@
       <c r="A783" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="B783" s="5" t="s">
+      <c r="B783" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C783" s="3"/>
@@ -10019,7 +10025,7 @@
       <c r="A784" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="B784" s="5" t="s">
+      <c r="B784" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C784" s="3"/>
@@ -10028,7 +10034,7 @@
       <c r="A785" s="1" t="s">
         <v>787</v>
       </c>
-      <c r="B785" s="5" t="s">
+      <c r="B785" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C785" s="3"/>
@@ -10037,7 +10043,7 @@
       <c r="A786" s="1" t="s">
         <v>788</v>
       </c>
-      <c r="B786" s="5" t="s">
+      <c r="B786" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C786" s="3"/>
@@ -10046,7 +10052,7 @@
       <c r="A787" s="1" t="s">
         <v>789</v>
       </c>
-      <c r="B787" s="5" t="s">
+      <c r="B787" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C787" s="3"/>
@@ -10055,7 +10061,7 @@
       <c r="A788" s="1" t="s">
         <v>790</v>
       </c>
-      <c r="B788" s="5" t="s">
+      <c r="B788" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C788" s="3"/>
@@ -10064,7 +10070,7 @@
       <c r="A789" s="1" t="s">
         <v>791</v>
       </c>
-      <c r="B789" s="5" t="s">
+      <c r="B789" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C789" s="3"/>
@@ -10073,7 +10079,7 @@
       <c r="A790" s="1" t="s">
         <v>792</v>
       </c>
-      <c r="B790" s="5" t="s">
+      <c r="B790" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C790" s="3"/>
@@ -10082,7 +10088,7 @@
       <c r="A791" s="1" t="s">
         <v>793</v>
       </c>
-      <c r="B791" s="5" t="s">
+      <c r="B791" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C791" s="3"/>
@@ -10091,7 +10097,7 @@
       <c r="A792" s="1" t="s">
         <v>794</v>
       </c>
-      <c r="B792" s="5" t="s">
+      <c r="B792" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C792" s="3"/>
@@ -10100,7 +10106,7 @@
       <c r="A793" s="1" t="s">
         <v>795</v>
       </c>
-      <c r="B793" s="5" t="s">
+      <c r="B793" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C793" s="3"/>
@@ -10109,7 +10115,7 @@
       <c r="A794" s="1" t="s">
         <v>796</v>
       </c>
-      <c r="B794" s="5" t="s">
+      <c r="B794" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C794" s="3"/>
@@ -10118,7 +10124,7 @@
       <c r="A795" s="1" t="s">
         <v>797</v>
       </c>
-      <c r="B795" s="5" t="s">
+      <c r="B795" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C795" s="3"/>
@@ -10127,7 +10133,7 @@
       <c r="A796" s="1" t="s">
         <v>798</v>
       </c>
-      <c r="B796" s="5" t="s">
+      <c r="B796" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C796" s="3"/>
@@ -10136,7 +10142,7 @@
       <c r="A797" s="1" t="s">
         <v>799</v>
       </c>
-      <c r="B797" s="5" t="s">
+      <c r="B797" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C797" s="3"/>
@@ -10145,7 +10151,7 @@
       <c r="A798" s="1" t="s">
         <v>800</v>
       </c>
-      <c r="B798" s="5" t="s">
+      <c r="B798" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C798" s="3"/>
@@ -10154,7 +10160,7 @@
       <c r="A799" s="1" t="s">
         <v>801</v>
       </c>
-      <c r="B799" s="5" t="s">
+      <c r="B799" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C799" s="3"/>
@@ -10163,7 +10169,7 @@
       <c r="A800" s="1" t="s">
         <v>802</v>
       </c>
-      <c r="B800" s="5" t="s">
+      <c r="B800" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C800" s="3"/>
@@ -10172,7 +10178,7 @@
       <c r="A801" s="1" t="s">
         <v>803</v>
       </c>
-      <c r="B801" s="5" t="s">
+      <c r="B801" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C801" s="3"/>
@@ -10181,7 +10187,7 @@
       <c r="A802" s="1" t="s">
         <v>804</v>
       </c>
-      <c r="B802" s="5" t="s">
+      <c r="B802" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C802" s="3"/>
@@ -10190,7 +10196,7 @@
       <c r="A803" s="1" t="s">
         <v>805</v>
       </c>
-      <c r="B803" s="5" t="s">
+      <c r="B803" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C803" s="3"/>
@@ -10199,7 +10205,7 @@
       <c r="A804" s="1" t="s">
         <v>806</v>
       </c>
-      <c r="B804" s="5" t="s">
+      <c r="B804" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C804" s="3"/>
@@ -10208,215 +10214,255 @@
       <c r="A805" s="1" t="s">
         <v>807</v>
       </c>
-      <c r="B805" s="5" t="s">
+      <c r="B805" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C805" s="3"/>
     </row>
     <row r="806" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A806" s="1"/>
-      <c r="B806" s="5" t="s">
+      <c r="B806" s="1" t="s">
         <v>808</v>
       </c>
       <c r="C806" s="3"/>
     </row>
     <row r="807" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A807" s="6" t="s">
+      <c r="A807" s="5" t="s">
         <v>809</v>
       </c>
-      <c r="B807" s="5" t="s">
+      <c r="B807" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C807" s="3"/>
     </row>
     <row r="808" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A808" s="6" t="s">
+      <c r="A808" s="5" t="s">
         <v>810</v>
       </c>
-      <c r="B808" s="5" t="s">
+      <c r="B808" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C808" s="3"/>
     </row>
     <row r="809" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A809" s="6" t="s">
+      <c r="A809" s="5" t="s">
         <v>811</v>
       </c>
-      <c r="B809" s="5" t="s">
+      <c r="B809" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C809" s="3"/>
     </row>
     <row r="810" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A810" s="6" t="s">
+      <c r="A810" s="5" t="s">
         <v>812</v>
       </c>
-      <c r="B810" s="5" t="s">
+      <c r="B810" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C810" s="3"/>
     </row>
     <row r="811" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A811" s="6" t="s">
+      <c r="A811" s="5" t="s">
         <v>813</v>
       </c>
-      <c r="B811" s="5" t="s">
+      <c r="B811" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C811" s="3"/>
     </row>
     <row r="812" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A812" s="6" t="s">
+      <c r="A812" s="5" t="s">
         <v>814</v>
       </c>
-      <c r="B812" s="5" t="s">
+      <c r="B812" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C812" s="3"/>
     </row>
     <row r="813" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A813" s="6" t="s">
+      <c r="A813" s="5" t="s">
         <v>815</v>
       </c>
-      <c r="B813" s="5" t="s">
+      <c r="B813" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C813" s="3"/>
     </row>
     <row r="814" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A814" s="6" t="s">
+      <c r="A814" s="5" t="s">
         <v>816</v>
       </c>
-      <c r="B814" s="5" t="s">
+      <c r="B814" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C814" s="3"/>
     </row>
     <row r="815" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A815" s="6" t="s">
+      <c r="A815" s="5" t="s">
         <v>817</v>
       </c>
-      <c r="B815" s="5" t="s">
+      <c r="B815" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C815" s="3"/>
     </row>
     <row r="816" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A816" s="6" t="s">
+      <c r="A816" s="5" t="s">
         <v>818</v>
       </c>
-      <c r="B816" s="5" t="s">
+      <c r="B816" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C816" s="3"/>
     </row>
     <row r="817" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A817" s="6" t="s">
+      <c r="A817" s="5" t="s">
         <v>819</v>
       </c>
-      <c r="B817" s="5" t="s">
+      <c r="B817" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C817" s="3"/>
     </row>
     <row r="818" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A818" s="6" t="s">
+      <c r="A818" s="5" t="s">
         <v>820</v>
       </c>
-      <c r="B818" s="5" t="s">
+      <c r="B818" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C818" s="3"/>
     </row>
     <row r="819" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A819" s="6" t="s">
+      <c r="A819" s="5" t="s">
         <v>821</v>
       </c>
-      <c r="B819" s="5" t="s">
+      <c r="B819" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C819" s="3"/>
     </row>
     <row r="820" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A820" s="6" t="s">
+      <c r="A820" s="5" t="s">
         <v>822</v>
       </c>
-      <c r="B820" s="5" t="s">
+      <c r="B820" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C820" s="3"/>
     </row>
     <row r="821" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A821" s="6" t="s">
+      <c r="A821" s="5" t="s">
         <v>823</v>
       </c>
-      <c r="B821" s="5" t="s">
+      <c r="B821" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C821" s="3"/>
     </row>
     <row r="822" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A822" s="6" t="s">
+      <c r="A822" s="5" t="s">
         <v>824</v>
       </c>
-      <c r="B822" s="5" t="s">
+      <c r="B822" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C822" s="3"/>
     </row>
     <row r="823" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A823" s="6" t="s">
+      <c r="A823" s="5" t="s">
         <v>825</v>
       </c>
-      <c r="B823" s="5" t="s">
+      <c r="B823" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C823" s="3"/>
     </row>
     <row r="824" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A824" s="6" t="s">
+      <c r="A824" s="5" t="s">
         <v>826</v>
       </c>
-      <c r="B824" s="5" t="s">
+      <c r="B824" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C824" s="3"/>
     </row>
     <row r="825" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A825" s="6" t="s">
+      <c r="A825" s="5" t="s">
         <v>827</v>
       </c>
-      <c r="B825" s="5" t="s">
+      <c r="B825" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C825" s="3"/>
     </row>
     <row r="826" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A826" s="6" t="s">
+      <c r="A826" s="5" t="s">
         <v>828</v>
       </c>
-      <c r="B826" s="5" t="s">
+      <c r="B826" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C826" s="3"/>
     </row>
     <row r="827" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A827" s="6" t="s">
+      <c r="A827" s="5" t="s">
         <v>829</v>
       </c>
-      <c r="B827" s="5" t="s">
+      <c r="B827" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C827" s="3"/>
     </row>
     <row r="828" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A828" s="6" t="s">
+      <c r="A828" s="5" t="s">
         <v>830</v>
       </c>
-      <c r="B828" s="5" t="s">
+      <c r="B828" s="1" t="s">
         <v>831</v>
       </c>
       <c r="C828" s="3"/>
+    </row>
+    <row r="829" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A829" s="6" t="s">
+        <v>832</v>
+      </c>
+      <c r="B829" s="1" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="830" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A830" s="6" t="s">
+        <v>833</v>
+      </c>
+      <c r="B830" s="1" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="831" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A831" s="6" t="s">
+        <v>834</v>
+      </c>
+      <c r="B831" s="1" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="832" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A832" s="6" t="s">
+        <v>835</v>
+      </c>
+      <c r="B832" s="1" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="833" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A833" s="6" t="s">
+        <v>836</v>
+      </c>
+      <c r="B833" s="1" t="s">
+        <v>831</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>